<commit_message>
Update GraphExcel.xlsx in FGNN/Data
</commit_message>
<xml_diff>
--- a/Data/GraphExcel.xlsx
+++ b/Data/GraphExcel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/qusai/Desktop/FGNN/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53B48F90-91FC-AE42-89AC-08E53AA079E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC236A60-2305-2445-B428-CFB69520357B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34200" yWindow="500" windowWidth="38400" windowHeight="23500" xr2:uid="{843B42F4-DAB3-4F48-AB22-1B3E609ACD3D}"/>
+    <workbookView xWindow="0" yWindow="880" windowWidth="34200" windowHeight="19660" xr2:uid="{843B42F4-DAB3-4F48-AB22-1B3E609ACD3D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2718" uniqueCount="1693">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2730" uniqueCount="1702">
   <si>
     <t xml:space="preserve"> p1              </t>
   </si>
@@ -5115,6 +5115,33 @@
   </si>
   <si>
     <t>Node2</t>
+  </si>
+  <si>
+    <t>PRV-1</t>
+  </si>
+  <si>
+    <t>n303</t>
+  </si>
+  <si>
+    <t>PRV-3</t>
+  </si>
+  <si>
+    <t>n226</t>
+  </si>
+  <si>
+    <t>PRV-2</t>
+  </si>
+  <si>
+    <t>n111</t>
+  </si>
+  <si>
+    <t>n336</t>
+  </si>
+  <si>
+    <t>n54</t>
+  </si>
+  <si>
+    <t>PUMP_1</t>
   </si>
 </sst>
 </file>
@@ -5486,7 +5513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{968E4133-7C5B-CA45-9374-5EE8F5CE52D1}">
-  <dimension ref="A1:C906"/>
+  <dimension ref="A1:C910"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -15455,6 +15482,50 @@
         <v>675</v>
       </c>
     </row>
+    <row r="907" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A907" t="s">
+        <v>1693</v>
+      </c>
+      <c r="B907" t="s">
+        <v>431</v>
+      </c>
+      <c r="C907" t="s">
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="908" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A908" t="s">
+        <v>1695</v>
+      </c>
+      <c r="B908" t="s">
+        <v>1696</v>
+      </c>
+      <c r="C908" t="s">
+        <v>1335</v>
+      </c>
+    </row>
+    <row r="909" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A909" t="s">
+        <v>1697</v>
+      </c>
+      <c r="B909" t="s">
+        <v>1698</v>
+      </c>
+      <c r="C909" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="910" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A910" t="s">
+        <v>1701</v>
+      </c>
+      <c r="B910" t="s">
+        <v>536</v>
+      </c>
+      <c r="C910" t="s">
+        <v>1700</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>